<commit_message>
Refresh the calculated workbook after the scenario band fix
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/4-revenue-modeling/tools/Aurumix_Revenue_Model_calculated.xlsx
+++ b/deliverables/4-revenue-modeling/tools/Aurumix_Revenue_Model_calculated.xlsx
@@ -1054,7 +1054,7 @@
     <t xml:space="preserve">Programme manager share of interchange</t>
   </si>
   <si>
-    <t xml:space="preserve">SIZES THE LARGEST STREAM. No UAE/MENA figure is published. FLOOR IS 36% - take that into the sponsor conversation as the walk-away. TRIANGULATED.</t>
+    <t xml:space="preserve">BANDS CORRECTED 2026-08-21 - THEY WERE INVERTED. Aggressive was 0.85 and conservative 0.55, meaning the OPTIMISTIC scenario handed MORE of the interchange to the programme manager and cut Aurumix's share from 28% to 15%. Every other cost-like parameter in this model improves under Aggressive - redemption, CAC, self-custody, the holder multiplier - and this one moved the other way. Flipping the scenario made interchange fall 46% in the good case and rise 61% in the bad one. Aggressive is now 0.36, THE DOCUMENTED FLOOR, which is the best deal observed anywhere and the right walk-away to take into a sponsor conversation - at that level Aurumix keeps 64% rather than 28%, and interchange more than doubles. Conservative is 0.85. WHY AURUMIX ONLY GETS A SLICE AT ALL: it is not a bank and cannot issue cards, so a programme manager holds the BIN, the scheme membership, settlement and dispute handling, and takes the majority for it. That much is normal. 72% is near the BAD END of the 36-85% range, so the base case is deliberately unfavourable - THIS IS A COMMERCIAL NEGOTIATION, NOT A MODELLING ASSUMPTION, and it is one of the few places where a better contract directly doubles a revenue line. No UAE/MENA figure is published. TRIANGULATED.</t>
   </si>
   <si>
     <t xml:space="preserve">Facility take-up - customers who take AND use the card</t>
@@ -6039,10 +6039,10 @@
         <v>0.72</v>
       </c>
       <c r="D44" s="19" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="E44" s="19" t="n">
         <v>0.85</v>
-      </c>
-      <c r="E44" s="19" t="n">
-        <v>0.55</v>
       </c>
       <c r="F44" s="23" t="s">
         <v>245</v>

</xml_diff>

<commit_message>
Refresh the calculated workbook after the interchange share change
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/4-revenue-modeling/tools/Aurumix_Revenue_Model_calculated.xlsx
+++ b/deliverables/4-revenue-modeling/tools/Aurumix_Revenue_Model_calculated.xlsx
@@ -1054,7 +1054,7 @@
     <t xml:space="preserve">Programme manager share of interchange</t>
   </si>
   <si>
-    <t xml:space="preserve">BANDS CORRECTED 2026-08-21 - THEY WERE INVERTED. Aggressive was 0.85 and conservative 0.55, meaning the OPTIMISTIC scenario handed MORE of the interchange to the programme manager and cut Aurumix's share from 28% to 15%. Every other cost-like parameter in this model improves under Aggressive - redemption, CAC, self-custody, the holder multiplier - and this one moved the other way. Flipping the scenario made interchange fall 46% in the good case and rise 61% in the bad one. Aggressive is now 0.36, THE DOCUMENTED FLOOR, which is the best deal observed anywhere and the right walk-away to take into a sponsor conversation - at that level Aurumix keeps 64% rather than 28%, and interchange more than doubles. Conservative is 0.85. WHY AURUMIX ONLY GETS A SLICE AT ALL: it is not a bank and cannot issue cards, so a programme manager holds the BIN, the scheme membership, settlement and dispute handling, and takes the majority for it. That much is normal. 72% is near the BAD END of the 36-85% range, so the base case is deliberately unfavourable - THIS IS A COMMERCIAL NEGOTIATION, NOT A MODELLING ASSUMPTION, and it is one of the few places where a better contract directly doubles a revenue line. No UAE/MENA figure is published. TRIANGULATED.</t>
+    <t xml:space="preserve">LOWERED 2026-08-21 from 0.72, client instruction - AURUMIX NOW KEEPS 40% RATHER THAN 28%. 0.60 sits comfortably inside the 36-85% observed range and is roughly its midpoint, so the base case moves from the pessimistic end to a neutral one. It assumes a NEGOTIATED deal rather than a take-it-or-leave-it one, which is reasonable for a programme with a gold-collateral proposition the manager cannot source elsewhere - but it IS an assumption about a contract that does not exist yet, and the only honest way to hold it is to treat 40% as a target to negotiate to, not a rate already won. BANDS CORRECTED earlier the same day - THEY WERE INVERTED. Aggressive was 0.85 and conservative 0.55, meaning the OPTIMISTIC scenario handed MORE of the interchange to the programme manager and cut Aurumix's share from 28% to 15%. Every other cost-like parameter in this model improves under Aggressive - redemption, CAC, self-custody, the holder multiplier - and this one moved the other way. Flipping the scenario made interchange fall 46% in the good case and rise 61% in the bad one. Aggressive is now 0.36, THE DOCUMENTED FLOOR, which is the best deal observed anywhere and the right walk-away to take into a sponsor conversation - at that level Aurumix keeps 64% rather than 28%, and interchange more than doubles. Conservative is 0.85. WHY AURUMIX ONLY GETS A SLICE AT ALL: it is not a bank and cannot issue cards, so a programme manager holds the BIN, the scheme membership, settlement and dispute handling, and takes the majority for it. That much is normal. 72% is near the BAD END of the 36-85% range, so the base case is deliberately unfavourable - THIS IS A COMMERCIAL NEGOTIATION, NOT A MODELLING ASSUMPTION, and it is one of the few places where a better contract directly doubles a revenue line. No UAE/MENA figure is published. TRIANGULATED.</t>
   </si>
   <si>
     <t xml:space="preserve">Facility take-up - customers who take AND use the card</t>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="B142" s="34" t="n">
         <f aca="false">'Scenario Parameters'!$B$44</f>
-        <v>0.72</v>
+        <v>0.6</v>
       </c>
       <c r="C142" s="0" t="s">
         <v>245</v>
@@ -6033,10 +6033,10 @@
       </c>
       <c r="B44" s="40" t="n">
         <f aca="false">CHOOSE($C$6,C44,D44,E44)</f>
-        <v>0.72</v>
+        <v>0.6</v>
       </c>
       <c r="C44" s="19" t="n">
-        <v>0.72</v>
+        <v>0.6</v>
       </c>
       <c r="D44" s="19" t="n">
         <v>0.36</v>
@@ -12512,71 +12512,71 @@
       </c>
       <c r="O56" s="55" t="n">
         <f aca="false">O51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>1.63946438106254</v>
+        <v>2.34209197294648</v>
       </c>
       <c r="P56" s="55" t="n">
         <f aca="false">P51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>1.69616037012857</v>
+        <v>2.42308624304082</v>
       </c>
       <c r="Q56" s="55" t="n">
         <f aca="false">Q51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>1.90552982178332</v>
+        <v>2.72218545969046</v>
       </c>
       <c r="R56" s="55" t="n">
         <f aca="false">R51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>2.12646524360413</v>
+        <v>3.03780749086304</v>
       </c>
       <c r="S56" s="55" t="n">
         <f aca="false">S51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>2.48672767906611</v>
+        <v>3.55246811295158</v>
       </c>
       <c r="T56" s="55" t="n">
         <f aca="false">T51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>2.82511939861288</v>
+        <v>4.03588485516125</v>
       </c>
       <c r="U56" s="55" t="n">
         <f aca="false">U51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>3.05503714664227</v>
+        <v>4.36433878091753</v>
       </c>
       <c r="V56" s="55" t="n">
         <f aca="false">V51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>3.55688213782489</v>
+        <v>5.08126019689269</v>
       </c>
       <c r="W56" s="55" t="n">
         <f aca="false">W51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>5.25235239439205</v>
+        <v>7.50336056341721</v>
       </c>
       <c r="X56" s="55" t="n">
         <f aca="false">X51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>6.58289875184579</v>
+        <v>9.40414107406541</v>
       </c>
       <c r="Y56" s="55" t="n">
         <f aca="false">Y51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>8.13192298401265</v>
+        <v>11.6170328343038</v>
       </c>
       <c r="Z56" s="55" t="n">
         <f aca="false">Z51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>10.8371945463668</v>
+        <v>15.4817064948096</v>
       </c>
       <c r="AA56" s="55" t="n">
         <f aca="false">AA51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>910.258390023829</v>
+        <v>1300.36912860547</v>
       </c>
       <c r="AB56" s="55" t="n">
         <f aca="false">AB51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>1990.88891248501</v>
+        <v>2844.12701783573</v>
       </c>
       <c r="AC56" s="55" t="n">
         <f aca="false">AC51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>3582.78438349205</v>
+        <v>5118.26340498864</v>
       </c>
       <c r="AD56" s="55" t="n">
         <f aca="false">AD51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>5624.33218013085</v>
+        <v>8034.76025732979</v>
       </c>
       <c r="AE56" s="55" t="n">
         <f aca="false">AE51*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>7925.24479729131</v>
+        <v>11321.7782818447</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13380,71 +13380,71 @@
       </c>
       <c r="O63" s="57" t="n">
         <f aca="false">O54+O55+O56+O58+O59+O61</f>
-        <v>2302.97612126652</v>
+        <v>2303.6787488584</v>
       </c>
       <c r="P63" s="57" t="n">
         <f aca="false">P54+P55+P56+P58+P59+P61</f>
-        <v>2861.60408394796</v>
+        <v>2862.33100982087</v>
       </c>
       <c r="Q63" s="57" t="n">
         <f aca="false">Q54+Q55+Q56+Q58+Q59+Q61</f>
-        <v>3376.25499123492</v>
+        <v>3377.07164687283</v>
       </c>
       <c r="R63" s="57" t="n">
         <f aca="false">R54+R55+R56+R58+R59+R61</f>
-        <v>4039.60702424243</v>
+        <v>4040.51836648969</v>
       </c>
       <c r="S63" s="57" t="n">
         <f aca="false">S54+S55+S56+S58+S59+S61</f>
-        <v>4609.85148485446</v>
+        <v>4610.91722528834</v>
       </c>
       <c r="T63" s="57" t="n">
         <f aca="false">T54+T55+T56+T58+T59+T61</f>
-        <v>5055.96210472257</v>
+        <v>5057.17287017911</v>
       </c>
       <c r="U63" s="57" t="n">
         <f aca="false">U54+U55+U56+U58+U59+U61</f>
-        <v>5462.50451002751</v>
+        <v>5463.81381166178</v>
       </c>
       <c r="V63" s="57" t="n">
         <f aca="false">V54+V55+V56+V58+V59+V61</f>
-        <v>5853.44125059046</v>
+        <v>5854.96562864952</v>
       </c>
       <c r="W63" s="57" t="n">
         <f aca="false">W54+W55+W56+W58+W59+W61</f>
-        <v>6351.90040462269</v>
+        <v>6354.15141279172</v>
       </c>
       <c r="X63" s="57" t="n">
         <f aca="false">X54+X55+X56+X58+X59+X61</f>
-        <v>7090.32092504897</v>
+        <v>7093.14216737119</v>
       </c>
       <c r="Y63" s="57" t="n">
         <f aca="false">Y54+Y55+Y56+Y58+Y59+Y61</f>
-        <v>7731.13243038532</v>
+        <v>7734.61754023561</v>
       </c>
       <c r="Z63" s="57" t="n">
         <f aca="false">Z54+Z55+Z56+Z58+Z59+Z61</f>
-        <v>8264.13584310114</v>
+        <v>8268.78035504959</v>
       </c>
       <c r="AA63" s="57" t="n">
         <f aca="false">AA54+AA55+AA56+AA58+AA59+AA61</f>
-        <v>220700.02638662</v>
+        <v>221090.137125202</v>
       </c>
       <c r="AB63" s="57" t="n">
         <f aca="false">AB54+AB55+AB56+AB58+AB59+AB61</f>
-        <v>378317.678400733</v>
+        <v>379170.916506084</v>
       </c>
       <c r="AC63" s="57" t="n">
         <f aca="false">AC54+AC55+AC56+AC58+AC59+AC61</f>
-        <v>581187.606379716</v>
+        <v>582723.085401212</v>
       </c>
       <c r="AD63" s="57" t="n">
         <f aca="false">AD54+AD55+AD56+AD58+AD59+AD61</f>
-        <v>785277.681872278</v>
+        <v>787688.109949477</v>
       </c>
       <c r="AE63" s="57" t="n">
         <f aca="false">AE54+AE55+AE56+AE58+AE59+AE61</f>
-        <v>949662.795101751</v>
+        <v>953059.328586305</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17289,39 +17289,39 @@
       </c>
       <c r="W96" s="55" t="n">
         <f aca="false">W91*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>0.172688951734677</v>
+        <v>0.24669850247811</v>
       </c>
       <c r="X96" s="55" t="n">
         <f aca="false">X91*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>0.36367872538033</v>
+        <v>0.519541036257614</v>
       </c>
       <c r="Y96" s="55" t="n">
         <f aca="false">Y91*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>0.587137418439322</v>
+        <v>0.838767740627603</v>
       </c>
       <c r="Z96" s="55" t="n">
         <f aca="false">Z91*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>0.961681791045065</v>
+        <v>1.37383113006438</v>
       </c>
       <c r="AA96" s="55" t="n">
         <f aca="false">AA91*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>166.863963083519</v>
+        <v>238.377090119313</v>
       </c>
       <c r="AB96" s="55" t="n">
         <f aca="false">AB91*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>392.845175697338</v>
+        <v>561.20739385334</v>
       </c>
       <c r="AC96" s="55" t="n">
         <f aca="false">AC91*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>727.997549931585</v>
+        <v>1039.99649990226</v>
       </c>
       <c r="AD96" s="55" t="n">
         <f aca="false">AD91*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>1158.1335047371</v>
+        <v>1654.47643533872</v>
       </c>
       <c r="AE96" s="55" t="n">
         <f aca="false">AE91*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>1638.08576322009</v>
+        <v>2340.12251888585</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18157,39 +18157,39 @@
       </c>
       <c r="W103" s="57" t="n">
         <f aca="false">W94+W95+W96+W98+W99+W101</f>
-        <v>1155.76359903911</v>
+        <v>1155.83760858985</v>
       </c>
       <c r="X103" s="57" t="n">
         <f aca="false">X94+X95+X96+X98+X99+X101</f>
-        <v>1340.89172276463</v>
+        <v>1341.04758507551</v>
       </c>
       <c r="Y103" s="57" t="n">
         <f aca="false">Y94+Y95+Y96+Y98+Y99+Y101</f>
-        <v>1503.36219445377</v>
+        <v>1503.61382477596</v>
       </c>
       <c r="Z103" s="57" t="n">
         <f aca="false">Z94+Z95+Z96+Z98+Z99+Z101</f>
-        <v>1641.67585734232</v>
+        <v>1642.08800668134</v>
       </c>
       <c r="AA103" s="57" t="n">
         <f aca="false">AA94+AA95+AA96+AA98+AA99+AA101</f>
-        <v>49257.4518417325</v>
+        <v>49328.9649687683</v>
       </c>
       <c r="AB103" s="57" t="n">
         <f aca="false">AB94+AB95+AB96+AB98+AB99+AB101</f>
-        <v>87121.5995334432</v>
+        <v>87289.9617515992</v>
       </c>
       <c r="AC103" s="57" t="n">
         <f aca="false">AC94+AC95+AC96+AC98+AC99+AC101</f>
-        <v>135243.911148384</v>
+        <v>135555.910098355</v>
       </c>
       <c r="AD103" s="57" t="n">
         <f aca="false">AD94+AD95+AD96+AD98+AD99+AD101</f>
-        <v>183529.982111776</v>
+        <v>184026.325042377</v>
       </c>
       <c r="AE103" s="57" t="n">
         <f aca="false">AE94+AE95+AE96+AE98+AE99+AE101</f>
-        <v>221021.19241832</v>
+        <v>221723.229173986</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22002,71 +22002,71 @@
       </c>
       <c r="O136" s="55" t="n">
         <f aca="false">O131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>3.2265946766555</v>
+        <v>4.60942096665072</v>
       </c>
       <c r="P136" s="55" t="n">
         <f aca="false">P131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>3.34415160271667</v>
+        <v>4.77735943245239</v>
       </c>
       <c r="Q136" s="55" t="n">
         <f aca="false">Q131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>3.75959810218154</v>
+        <v>5.37085443168792</v>
       </c>
       <c r="R136" s="55" t="n">
         <f aca="false">R131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>4.198222212821</v>
+        <v>5.99746030403001</v>
       </c>
       <c r="S136" s="55" t="n">
         <f aca="false">S131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>4.90936976293557</v>
+        <v>7.01338537562224</v>
       </c>
       <c r="T136" s="55" t="n">
         <f aca="false">T131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>5.57427259767526</v>
+        <v>7.96324656810751</v>
       </c>
       <c r="U136" s="55" t="n">
         <f aca="false">U131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>6.02456762531877</v>
+        <v>8.60652517902681</v>
       </c>
       <c r="V136" s="55" t="n">
         <f aca="false">V131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>7.01103927228932</v>
+        <v>10.0157703889847</v>
       </c>
       <c r="W136" s="55" t="n">
         <f aca="false">W131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>10.2950862515356</v>
+        <v>14.7072660736222</v>
       </c>
       <c r="X136" s="55" t="n">
         <f aca="false">X131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>12.858510220029</v>
+        <v>18.3693003143271</v>
       </c>
       <c r="Y136" s="55" t="n">
         <f aca="false">Y131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>15.8386085395762</v>
+        <v>22.626583627966</v>
       </c>
       <c r="Z136" s="55" t="n">
         <f aca="false">Z131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>21.0368879241544</v>
+        <v>30.0526970345063</v>
       </c>
       <c r="AA136" s="55" t="n">
         <f aca="false">AA131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>1600.54171459423</v>
+        <v>2286.48816370604</v>
       </c>
       <c r="AB136" s="55" t="n">
         <f aca="false">AB131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>3312.45563186364</v>
+        <v>4732.07947409092</v>
       </c>
       <c r="AC136" s="55" t="n">
         <f aca="false">AC131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>5584.83444236091</v>
+        <v>7978.33491765845</v>
       </c>
       <c r="AD136" s="55" t="n">
         <f aca="false">AD131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>8108.09316038188</v>
+        <v>11582.990229117</v>
       </c>
       <c r="AE136" s="55" t="n">
         <f aca="false">AE131*IF(Assumptions!$B$178=1,MIN(Assumptions!$B$14,1%),Assumptions!$B$14)*(1-Assumptions!$B$142)</f>
-        <v>10383.7583082959</v>
+        <v>14833.9404404227</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22870,71 +22870,71 @@
       </c>
       <c r="O143" s="57" t="n">
         <f aca="false">O134+O135+O136+O138+O139+O141</f>
-        <v>4625.19209695194</v>
+        <v>4626.57492324194</v>
       </c>
       <c r="P143" s="57" t="n">
         <f aca="false">P134+P135+P136+P138+P139+P141</f>
-        <v>5729.84813882029</v>
+        <v>5731.28134665002</v>
       </c>
       <c r="Q143" s="57" t="n">
         <f aca="false">Q134+Q135+Q136+Q138+Q139+Q141</f>
-        <v>6742.74208501814</v>
+        <v>6744.35334134765</v>
       </c>
       <c r="R143" s="57" t="n">
         <f aca="false">R134+R135+R136+R138+R139+R141</f>
-        <v>8042.98552207297</v>
+        <v>8044.78476016418</v>
       </c>
       <c r="S143" s="57" t="n">
         <f aca="false">S134+S135+S136+S138+S139+S141</f>
-        <v>9154.22461298518</v>
+        <v>9156.32862859787</v>
       </c>
       <c r="T143" s="57" t="n">
         <f aca="false">T134+T135+T136+T138+T139+T141</f>
-        <v>10019.5823257497</v>
+        <v>10021.9712997202</v>
       </c>
       <c r="U143" s="57" t="n">
         <f aca="false">U134+U135+U136+U138+U139+U141</f>
-        <v>10802.8258004017</v>
+        <v>10805.4077579554</v>
       </c>
       <c r="V143" s="57" t="n">
         <f aca="false">V134+V135+V136+V138+V139+V141</f>
-        <v>11550.6574237996</v>
+        <v>11553.6621549163</v>
       </c>
       <c r="W143" s="57" t="n">
         <f aca="false">W134+W135+W136+W138+W139+W141</f>
-        <v>12514.7343302613</v>
+        <v>12519.1465100833</v>
       </c>
       <c r="X143" s="57" t="n">
         <f aca="false">X134+X135+X136+X138+X139+X141</f>
-        <v>13933.373119992</v>
+        <v>13938.8839100863</v>
       </c>
       <c r="Y143" s="57" t="n">
         <f aca="false">Y134+Y135+Y136+Y138+Y139+Y141</f>
-        <v>15153.9086340652</v>
+        <v>15160.6966091536</v>
       </c>
       <c r="Z143" s="57" t="n">
         <f aca="false">Z134+Z135+Z136+Z138+Z139+Z141</f>
-        <v>16165.2349362255</v>
+        <v>16174.2507453358</v>
       </c>
       <c r="AA143" s="57" t="n">
         <f aca="false">AA134+AA135+AA136+AA138+AA139+AA141</f>
-        <v>398267.480972361</v>
+        <v>398953.427421473</v>
       </c>
       <c r="AB143" s="57" t="n">
         <f aca="false">AB134+AB135+AB136+AB138+AB139+AB141</f>
-        <v>638803.042779799</v>
+        <v>640222.666622026</v>
       </c>
       <c r="AC143" s="57" t="n">
         <f aca="false">AC134+AC135+AC136+AC138+AC139+AC141</f>
-        <v>895641.010552015</v>
+        <v>898034.511027313</v>
       </c>
       <c r="AD143" s="57" t="n">
         <f aca="false">AD134+AD135+AD136+AD138+AD139+AD141</f>
-        <v>1075704.63157371</v>
+        <v>1079179.52864244</v>
       </c>
       <c r="AE143" s="57" t="n">
         <f aca="false">AE134+AE135+AE136+AE138+AE139+AE141</f>
-        <v>1107734.71391493</v>
+        <v>1112184.89604705</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26179,71 +26179,71 @@
       </c>
       <c r="O177" s="55" t="n">
         <f aca="false">O56+O96+O136</f>
-        <v>4.86605905771804</v>
+        <v>6.95151293959719</v>
       </c>
       <c r="P177" s="55" t="n">
         <f aca="false">P56+P96+P136</f>
-        <v>5.04031197284524</v>
+        <v>7.2004456754932</v>
       </c>
       <c r="Q177" s="55" t="n">
         <f aca="false">Q56+Q96+Q136</f>
-        <v>5.66512792396486</v>
+        <v>8.09303989137838</v>
       </c>
       <c r="R177" s="55" t="n">
         <f aca="false">R56+R96+R136</f>
-        <v>6.32468745642513</v>
+        <v>9.03526779489304</v>
       </c>
       <c r="S177" s="55" t="n">
         <f aca="false">S56+S96+S136</f>
-        <v>7.39609744200167</v>
+        <v>10.5658534885738</v>
       </c>
       <c r="T177" s="55" t="n">
         <f aca="false">T56+T96+T136</f>
-        <v>8.39939199628813</v>
+        <v>11.9991314232688</v>
       </c>
       <c r="U177" s="55" t="n">
         <f aca="false">U56+U96+U136</f>
-        <v>9.07960477196104</v>
+        <v>12.9708639599443</v>
       </c>
       <c r="V177" s="55" t="n">
         <f aca="false">V56+V96+V136</f>
-        <v>10.5679214101142</v>
+        <v>15.0970305858774</v>
       </c>
       <c r="W177" s="55" t="n">
         <f aca="false">W56+W96+W136</f>
-        <v>15.7201275976623</v>
+        <v>22.4573251395176</v>
       </c>
       <c r="X177" s="55" t="n">
         <f aca="false">X56+X96+X136</f>
-        <v>19.8050876972551</v>
+        <v>28.2929824246501</v>
       </c>
       <c r="Y177" s="55" t="n">
         <f aca="false">Y56+Y96+Y136</f>
-        <v>24.5576689420282</v>
+        <v>35.0823842028974</v>
       </c>
       <c r="Z177" s="55" t="n">
         <f aca="false">Z56+Z96+Z136</f>
-        <v>32.8357642615662</v>
+        <v>46.9082346593803</v>
       </c>
       <c r="AA177" s="55" t="n">
         <f aca="false">AA56+AA96+AA136</f>
-        <v>2677.66406770158</v>
+        <v>3825.23438243083</v>
       </c>
       <c r="AB177" s="55" t="n">
         <f aca="false">AB56+AB96+AB136</f>
-        <v>5696.18972004599</v>
+        <v>8137.41388577998</v>
       </c>
       <c r="AC177" s="55" t="n">
         <f aca="false">AC56+AC96+AC136</f>
-        <v>9895.61637578455</v>
+        <v>14136.5948225494</v>
       </c>
       <c r="AD177" s="55" t="n">
         <f aca="false">AD56+AD96+AD136</f>
-        <v>14890.5588452498</v>
+        <v>21272.2269217855</v>
       </c>
       <c r="AE177" s="55" t="n">
         <f aca="false">AE56+AE96+AE136</f>
-        <v>19947.0888688073</v>
+        <v>28495.8412411533</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26923,71 +26923,71 @@
       </c>
       <c r="O183" s="57" t="n">
         <f aca="false">O63+O103+O143+O147</f>
-        <v>18891.2849425638</v>
+        <v>18893.3703964457</v>
       </c>
       <c r="P183" s="57" t="n">
         <f aca="false">P63+P103+P143+P147</f>
-        <v>20693.3240226263</v>
+        <v>20695.484156329</v>
       </c>
       <c r="Q183" s="57" t="n">
         <f aca="false">Q63+Q103+Q143+Q147</f>
-        <v>22349.2922546306</v>
+        <v>22351.720166598</v>
       </c>
       <c r="R183" s="57" t="n">
         <f aca="false">R63+R103+R143+R147</f>
-        <v>24474.4495136757</v>
+        <v>24477.1600940142</v>
       </c>
       <c r="S183" s="57" t="n">
         <f aca="false">S63+S103+S143+S147</f>
-        <v>26295.4591064206</v>
+        <v>26298.6288624672</v>
       </c>
       <c r="T183" s="57" t="n">
         <f aca="false">T63+T103+T143+T147</f>
-        <v>27715.6303800683</v>
+        <v>27719.2301194953</v>
       </c>
       <c r="U183" s="57" t="n">
         <f aca="false">U63+U103+U143+U147</f>
-        <v>29005.5831057585</v>
+        <v>29009.4743649465</v>
       </c>
       <c r="V183" s="57" t="n">
         <f aca="false">V63+V103+V143+V147</f>
-        <v>30241.3416662486</v>
+        <v>30245.8707754243</v>
       </c>
       <c r="W183" s="57" t="n">
         <f aca="false">W63+W103+W143+W147</f>
-        <v>31834.8983339231</v>
+        <v>31841.6355314649</v>
       </c>
       <c r="X183" s="57" t="n">
         <f aca="false">X63+X103+X143+X147</f>
-        <v>34177.0857678056</v>
+        <v>34185.573662533</v>
       </c>
       <c r="Y183" s="57" t="n">
         <f aca="false">Y63+Y103+Y143+Y147</f>
-        <v>36200.9032589043</v>
+        <v>36211.4279741651</v>
       </c>
       <c r="Z183" s="57" t="n">
         <f aca="false">Z63+Z103+Z143+Z147</f>
-        <v>37883.546636669</v>
+        <v>37897.6191070668</v>
       </c>
       <c r="AA183" s="57" t="n">
         <f aca="false">AA63+AA103+AA143+AA147</f>
-        <v>1093474.95920071</v>
+        <v>1094622.52951544</v>
       </c>
       <c r="AB183" s="57" t="n">
         <f aca="false">AB63+AB103+AB143+AB147</f>
-        <v>1812992.32071398</v>
+        <v>1815433.54487971</v>
       </c>
       <c r="AC183" s="57" t="n">
         <f aca="false">AC63+AC103+AC143+AC147</f>
-        <v>2604322.52808011</v>
+        <v>2608563.50652688</v>
       </c>
       <c r="AD183" s="57" t="n">
         <f aca="false">AD63+AD103+AD143+AD147</f>
-        <v>3320262.29555776</v>
+        <v>3326643.9636343</v>
       </c>
       <c r="AE183" s="57" t="n">
         <f aca="false">AE63+AE103+AE143+AE147</f>
-        <v>3837668.701435</v>
+        <v>3846217.45380734</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27047,71 +27047,71 @@
       </c>
       <c r="O184" s="55" t="n">
         <f aca="false">IF(O151=0,0,O183/O151/O7*12)</f>
-        <v>73.3043425747494</v>
+        <v>73.3124348154967</v>
       </c>
       <c r="P184" s="55" t="n">
         <f aca="false">IF(P151=0,0,P183/P151/P7*12)</f>
-        <v>65.010232184953</v>
+        <v>65.0170184699117</v>
       </c>
       <c r="Q184" s="55" t="n">
         <f aca="false">IF(Q151=0,0,Q183/Q151/Q7*12)</f>
-        <v>59.7073075775561</v>
+        <v>59.7137938718404</v>
       </c>
       <c r="R184" s="55" t="n">
         <f aca="false">IF(R151=0,0,R183/R151/R7*12)</f>
-        <v>54.7463127308284</v>
+        <v>54.7523759633767</v>
       </c>
       <c r="S184" s="55" t="n">
         <f aca="false">IF(S151=0,0,S183/S151/S7*12)</f>
-        <v>51.619494690748</v>
+        <v>51.6257171037036</v>
       </c>
       <c r="T184" s="55" t="n">
         <f aca="false">IF(T151=0,0,T183/T151/T7*12)</f>
-        <v>49.7490678791548</v>
+        <v>49.7555293479593</v>
       </c>
       <c r="U184" s="55" t="n">
         <f aca="false">IF(U151=0,0,U183/U151/U7*12)</f>
-        <v>48.2663442007566</v>
+        <v>48.2728193974336</v>
       </c>
       <c r="V184" s="55" t="n">
         <f aca="false">IF(V151=0,0,V183/V151/V7*12)</f>
-        <v>46.9959198131693</v>
+        <v>47.0029581798528</v>
       </c>
       <c r="W184" s="55" t="n">
         <f aca="false">IF(W151=0,0,W183/W151/W7*12)</f>
-        <v>46.0323458614957</v>
+        <v>46.0420876550498</v>
       </c>
       <c r="X184" s="55" t="n">
         <f aca="false">IF(X151=0,0,X183/X151/X7*12)</f>
-        <v>44.6209842469344</v>
+        <v>44.6320658885785</v>
       </c>
       <c r="Y184" s="55" t="n">
         <f aca="false">IF(Y151=0,0,Y183/Y151/Y7*12)</f>
-        <v>43.6173126609797</v>
+        <v>43.6299935544071</v>
       </c>
       <c r="Z184" s="55" t="n">
         <f aca="false">IF(Z151=0,0,Z183/Z151/Z7*12)</f>
-        <v>43.0523178803063</v>
+        <v>43.0683103763294</v>
       </c>
       <c r="AA184" s="55" t="n">
         <f aca="false">IF(AA151=0,0,AA183/AA151/AA7*12)</f>
-        <v>54.2484150253178</v>
+        <v>54.3053471664522</v>
       </c>
       <c r="AB184" s="55" t="n">
         <f aca="false">IF(AB151=0,0,AB183/AB151/AB7*12)</f>
-        <v>55.3427742349258</v>
+        <v>55.4172941963826</v>
       </c>
       <c r="AC184" s="55" t="n">
         <f aca="false">IF(AC151=0,0,AC183/AC151/AC7*12)</f>
-        <v>55.4386595608927</v>
+        <v>55.5289379952188</v>
       </c>
       <c r="AD184" s="55" t="n">
         <f aca="false">IF(AD151=0,0,AD183/AD151/AD7*12)</f>
-        <v>57.0713394473762</v>
+        <v>57.1810326922514</v>
       </c>
       <c r="AE184" s="55" t="n">
         <f aca="false">IF(AE151=0,0,AE183/AE151/AE7*12)</f>
-        <v>61.3054809929673</v>
+        <v>61.4420444685691</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27321,27 +27321,27 @@
       </c>
       <c r="E7" s="36" t="n">
         <f aca="false">SUM(Model!O63:Z63)</f>
-        <v>62999.6911740449</v>
+        <v>63021.1607832686</v>
       </c>
       <c r="F7" s="36" t="n">
         <f aca="false">Model!AA63</f>
-        <v>220700.02638662</v>
+        <v>221090.137125202</v>
       </c>
       <c r="G7" s="36" t="n">
         <f aca="false">Model!AB63</f>
-        <v>378317.678400733</v>
+        <v>379170.916506084</v>
       </c>
       <c r="H7" s="36" t="n">
         <f aca="false">Model!AC63</f>
-        <v>581187.606379716</v>
+        <v>582723.085401212</v>
       </c>
       <c r="I7" s="36" t="n">
         <f aca="false">Model!AD63</f>
-        <v>785277.681872278</v>
+        <v>787688.109949477</v>
       </c>
       <c r="J7" s="36" t="n">
         <f aca="false">Model!AE63</f>
-        <v>949662.795101751</v>
+        <v>953059.328586305</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27354,27 +27354,27 @@
       </c>
       <c r="E8" s="36" t="n">
         <f aca="false">SUM(Model!O103:Z103)</f>
-        <v>10577.7987889059</v>
+        <v>10578.6924404288</v>
       </c>
       <c r="F8" s="36" t="n">
         <f aca="false">Model!AA103</f>
-        <v>49257.4518417325</v>
+        <v>49328.9649687683</v>
       </c>
       <c r="G8" s="36" t="n">
         <f aca="false">Model!AB103</f>
-        <v>87121.5995334432</v>
+        <v>87289.9617515992</v>
       </c>
       <c r="H8" s="36" t="n">
         <f aca="false">Model!AC103</f>
-        <v>135243.911148384</v>
+        <v>135555.910098355</v>
       </c>
       <c r="I8" s="36" t="n">
         <f aca="false">Model!AD103</f>
-        <v>183529.982111776</v>
+        <v>184026.325042377</v>
       </c>
       <c r="J8" s="36" t="n">
         <f aca="false">Model!AE103</f>
-        <v>221021.19241832</v>
+        <v>221723.229173986</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27387,27 +27387,27 @@
       </c>
       <c r="E9" s="36" t="n">
         <f aca="false">SUM(Model!O143:Z143)</f>
-        <v>124435.309026343</v>
+        <v>124477.341987253</v>
       </c>
       <c r="F9" s="36" t="n">
         <f aca="false">Model!AA143</f>
-        <v>398267.480972361</v>
+        <v>398953.427421473</v>
       </c>
       <c r="G9" s="36" t="n">
         <f aca="false">Model!AB143</f>
-        <v>638803.042779799</v>
+        <v>640222.666622026</v>
       </c>
       <c r="H9" s="36" t="n">
         <f aca="false">Model!AC143</f>
-        <v>895641.010552015</v>
+        <v>898034.511027313</v>
       </c>
       <c r="I9" s="36" t="n">
         <f aca="false">Model!AD143</f>
-        <v>1075704.63157371</v>
+        <v>1079179.52864244</v>
       </c>
       <c r="J9" s="36" t="n">
         <f aca="false">Model!AE143</f>
-        <v>1107734.71391493</v>
+        <v>1112184.89604705</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27453,27 +27453,27 @@
       </c>
       <c r="E11" s="62" t="n">
         <f aca="false">SUM(Model!O183:Z183)</f>
-        <v>339762.798989294</v>
+        <v>339827.19521095</v>
       </c>
       <c r="F11" s="62" t="n">
         <f aca="false">Model!AA183</f>
-        <v>1093474.95920071</v>
+        <v>1094622.52951544</v>
       </c>
       <c r="G11" s="62" t="n">
         <f aca="false">Model!AB183</f>
-        <v>1812992.32071398</v>
+        <v>1815433.54487971</v>
       </c>
       <c r="H11" s="62" t="n">
         <f aca="false">Model!AC183</f>
-        <v>2604322.52808011</v>
+        <v>2608563.50652688</v>
       </c>
       <c r="I11" s="62" t="n">
         <f aca="false">Model!AD183</f>
-        <v>3320262.29555776</v>
+        <v>3326643.9636343</v>
       </c>
       <c r="J11" s="62" t="n">
         <f aca="false">Model!AE183</f>
-        <v>3837668.701435</v>
+        <v>3846217.45380734</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27567,27 +27567,27 @@
       </c>
       <c r="E16" s="36" t="n">
         <f aca="false">SUM(Model!O177:Z177)</f>
-        <v>150.25785052983</v>
+        <v>214.654072185472</v>
       </c>
       <c r="F16" s="36" t="n">
         <f aca="false">Model!AA177</f>
-        <v>2677.66406770158</v>
+        <v>3825.23438243083</v>
       </c>
       <c r="G16" s="36" t="n">
         <f aca="false">Model!AB177</f>
-        <v>5696.18972004599</v>
+        <v>8137.41388577998</v>
       </c>
       <c r="H16" s="36" t="n">
         <f aca="false">Model!AC177</f>
-        <v>9895.61637578455</v>
+        <v>14136.5948225494</v>
       </c>
       <c r="I16" s="36" t="n">
         <f aca="false">Model!AD177</f>
-        <v>14890.5588452498</v>
+        <v>21272.2269217855</v>
       </c>
       <c r="J16" s="36" t="n">
         <f aca="false">Model!AE177</f>
-        <v>19947.0888688073</v>
+        <v>28495.8412411533</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27732,27 +27732,27 @@
       </c>
       <c r="E21" s="62" t="n">
         <f aca="false">SUM(Model!O183:Z183)</f>
-        <v>339762.798989294</v>
+        <v>339827.19521095</v>
       </c>
       <c r="F21" s="62" t="n">
         <f aca="false">Model!AA183</f>
-        <v>1093474.95920071</v>
+        <v>1094622.52951544</v>
       </c>
       <c r="G21" s="62" t="n">
         <f aca="false">Model!AB183</f>
-        <v>1812992.32071398</v>
+        <v>1815433.54487971</v>
       </c>
       <c r="H21" s="62" t="n">
         <f aca="false">Model!AC183</f>
-        <v>2604322.52808011</v>
+        <v>2608563.50652688</v>
       </c>
       <c r="I21" s="62" t="n">
         <f aca="false">Model!AD183</f>
-        <v>3320262.29555776</v>
+        <v>3326643.9636343</v>
       </c>
       <c r="J21" s="62" t="n">
         <f aca="false">Model!AE183</f>
-        <v>3837668.701435</v>
+        <v>3846217.45380734</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27780,27 +27780,27 @@
       </c>
       <c r="E24" s="63" t="n">
         <f aca="false">IF(E$11=0,0,E14/E$11)</f>
-        <v>0.374253260671347</v>
+        <v>0.374182340814816</v>
       </c>
       <c r="F24" s="63" t="n">
         <f aca="false">IF(F$11=0,0,F14/F$11)</f>
-        <v>0.340508870642117</v>
+        <v>0.340151891079469</v>
       </c>
       <c r="G24" s="63" t="n">
         <f aca="false">IF(G$11=0,0,G14/G$11)</f>
-        <v>0.333998500987281</v>
+        <v>0.333549371238506</v>
       </c>
       <c r="H24" s="63" t="n">
         <f aca="false">IF(H$11=0,0,H14/H$11)</f>
-        <v>0.333879925769189</v>
+        <v>0.333337106870799</v>
       </c>
       <c r="I24" s="63" t="n">
         <f aca="false">IF(I$11=0,0,I14/I$11)</f>
-        <v>0.324966192894997</v>
+        <v>0.324342793937422</v>
       </c>
       <c r="J24" s="63" t="n">
         <f aca="false">IF(J$11=0,0,J14/J$11)</f>
-        <v>0.303428881638009</v>
+        <v>0.302754468814789</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27813,27 +27813,27 @@
       </c>
       <c r="E25" s="63" t="n">
         <f aca="false">IF(E$11=0,0,E15/E$11)</f>
-        <v>0.0286069917924122</v>
+        <v>0.0286015708543286</v>
       </c>
       <c r="F25" s="63" t="n">
         <f aca="false">IF(F$11=0,0,F15/F$11)</f>
-        <v>0.0262664180832223</v>
+        <v>0.0262388811370571</v>
       </c>
       <c r="G25" s="63" t="n">
         <f aca="false">IF(G$11=0,0,G15/G$11)</f>
-        <v>0.0259174954148117</v>
+        <v>0.0258826440062871</v>
       </c>
       <c r="H25" s="63" t="n">
         <f aca="false">IF(H$11=0,0,H15/H$11)</f>
-        <v>0.0261219531182726</v>
+        <v>0.0260794842882499</v>
       </c>
       <c r="I25" s="63" t="n">
         <f aca="false">IF(I$11=0,0,I15/I$11)</f>
-        <v>0.0257017173890064</v>
+        <v>0.0256524124945944</v>
       </c>
       <c r="J25" s="63" t="n">
         <f aca="false">IF(J$11=0,0,J15/J$11)</f>
-        <v>0.024368554846068</v>
+        <v>0.0243143923491336</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27846,27 +27846,27 @@
       </c>
       <c r="E26" s="63" t="n">
         <f aca="false">IF(E$11=0,0,E16/E$11)</f>
-        <v>0.000442243385611397</v>
+        <v>0.00063165654547519</v>
       </c>
       <c r="F26" s="63" t="n">
         <f aca="false">IF(F$11=0,0,F16/F$11)</f>
-        <v>0.00244876578578338</v>
+        <v>0.0034945693874254</v>
       </c>
       <c r="G26" s="63" t="n">
         <f aca="false">IF(G$11=0,0,G16/G$11)</f>
-        <v>0.00314187195111934</v>
+        <v>0.00448235293918135</v>
       </c>
       <c r="H26" s="63" t="n">
         <f aca="false">IF(H$11=0,0,H16/H$11)</f>
-        <v>0.00379968927392396</v>
+        <v>0.00541930253458588</v>
       </c>
       <c r="I26" s="63" t="n">
         <f aca="false">IF(I$11=0,0,I16/I$11)</f>
-        <v>0.00448475376935496</v>
+        <v>0.0063945006301624</v>
       </c>
       <c r="J26" s="63" t="n">
         <f aca="false">IF(J$11=0,0,J16/J$11)</f>
-        <v>0.00519770996942717</v>
+        <v>0.00740879619610313</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27879,27 +27879,27 @@
       </c>
       <c r="E27" s="63" t="n">
         <f aca="false">IF(E$11=0,0,E17/E$11)</f>
-        <v>0.144711341240812</v>
+        <v>0.144683918881042</v>
       </c>
       <c r="F27" s="63" t="n">
         <f aca="false">IF(F$11=0,0,F17/F$11)</f>
-        <v>0.129837499904932</v>
+        <v>0.12970138205918</v>
       </c>
       <c r="G27" s="63" t="n">
         <f aca="false">IF(G$11=0,0,G17/G$11)</f>
-        <v>0.123924339603843</v>
+        <v>0.123757697815485</v>
       </c>
       <c r="H27" s="63" t="n">
         <f aca="false">IF(H$11=0,0,H17/H$11)</f>
-        <v>0.120810417651675</v>
+        <v>0.1206140051909</v>
       </c>
       <c r="I27" s="63" t="n">
         <f aca="false">IF(I$11=0,0,I17/I$11)</f>
-        <v>0.113741232359714</v>
+        <v>0.113523036845114</v>
       </c>
       <c r="J27" s="63" t="n">
         <f aca="false">IF(J$11=0,0,J17/J$11)</f>
-        <v>0.101707860973294</v>
+        <v>0.101481801129246</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27912,27 +27912,27 @@
       </c>
       <c r="E28" s="63" t="n">
         <f aca="false">IF(E$11=0,0,E18/E$11)</f>
-        <v>0.0342699510347229</v>
+        <v>0.0342634569830577</v>
       </c>
       <c r="F28" s="63" t="n">
         <f aca="false">IF(F$11=0,0,F18/F$11)</f>
-        <v>0.109027743025992</v>
+        <v>0.108913441522044</v>
       </c>
       <c r="G28" s="63" t="n">
         <f aca="false">IF(G$11=0,0,G18/G$11)</f>
-        <v>0.118122626342778</v>
+        <v>0.117963786152367</v>
       </c>
       <c r="H28" s="63" t="n">
         <f aca="false">IF(H$11=0,0,H18/H$11)</f>
-        <v>0.129461693106865</v>
+        <v>0.129251215482389</v>
       </c>
       <c r="I28" s="63" t="n">
         <f aca="false">IF(I$11=0,0,I18/I$11)</f>
-        <v>0.140855383319811</v>
+        <v>0.140585173368591</v>
       </c>
       <c r="J28" s="63" t="n">
         <f aca="false">IF(J$11=0,0,J18/J$11)</f>
-        <v>0.151662674317086</v>
+        <v>0.151325582963715</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27945,27 +27945,27 @@
       </c>
       <c r="E29" s="63" t="n">
         <f aca="false">IF(E$11=0,0,E19/E$11)</f>
-        <v>0.000513385604328451</v>
+        <v>0.000513288319315253</v>
       </c>
       <c r="F29" s="63" t="n">
         <f aca="false">IF(F$11=0,0,F19/F$11)</f>
-        <v>0.00301290803429898</v>
+        <v>0.00300974938944384</v>
       </c>
       <c r="G29" s="63" t="n">
         <f aca="false">IF(G$11=0,0,G19/G$11)</f>
-        <v>0.00396686892674896</v>
+        <v>0.00396153465477101</v>
       </c>
       <c r="H29" s="63" t="n">
         <f aca="false">IF(H$11=0,0,H19/H$11)</f>
-        <v>0.00492512429993497</v>
+        <v>0.00491711707835443</v>
       </c>
       <c r="I29" s="63" t="n">
         <f aca="false">IF(I$11=0,0,I19/I$11)</f>
-        <v>0.00601902817855839</v>
+        <v>0.00600748157471417</v>
       </c>
       <c r="J29" s="63" t="n">
         <f aca="false">IF(J$11=0,0,J19/J$11)</f>
-        <v>0.00733296154521509</v>
+        <v>0.00731666301993438</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27978,27 +27978,27 @@
       </c>
       <c r="E30" s="63" t="n">
         <f aca="false">IF(E$11=0,0,E20/E$11)</f>
-        <v>0.417202826270767</v>
+        <v>0.417123767601965</v>
       </c>
       <c r="F30" s="63" t="n">
         <f aca="false">IF(F$11=0,0,F20/F$11)</f>
-        <v>0.388897794523654</v>
+        <v>0.38849008542538</v>
       </c>
       <c r="G30" s="63" t="n">
         <f aca="false">IF(G$11=0,0,G20/G$11)</f>
-        <v>0.390928296773418</v>
+        <v>0.390402613193402</v>
       </c>
       <c r="H30" s="63" t="n">
         <f aca="false">IF(H$11=0,0,H20/H$11)</f>
-        <v>0.381001196780139</v>
+        <v>0.380381768554721</v>
       </c>
       <c r="I30" s="63" t="n">
         <f aca="false">IF(I$11=0,0,I20/I$11)</f>
-        <v>0.384231692088558</v>
+        <v>0.383494601149402</v>
       </c>
       <c r="J30" s="63" t="n">
         <f aca="false">IF(J$11=0,0,J20/J$11)</f>
-        <v>0.406301356710901</v>
+        <v>0.405398295527079</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28356,27 +28356,27 @@
       </c>
       <c r="E43" s="36" t="n">
         <f aca="false">Model!Z184</f>
-        <v>43.0523178803063</v>
+        <v>43.0683103763294</v>
       </c>
       <c r="F43" s="36" t="n">
         <f aca="false">Model!AA184</f>
-        <v>54.2484150253178</v>
+        <v>54.3053471664522</v>
       </c>
       <c r="G43" s="36" t="n">
         <f aca="false">Model!AB184</f>
-        <v>55.3427742349258</v>
+        <v>55.4172941963826</v>
       </c>
       <c r="H43" s="36" t="n">
         <f aca="false">Model!AC184</f>
-        <v>55.4386595608927</v>
+        <v>55.5289379952188</v>
       </c>
       <c r="I43" s="36" t="n">
         <f aca="false">Model!AD184</f>
-        <v>57.0713394473762</v>
+        <v>57.1810326922514</v>
       </c>
       <c r="J43" s="36" t="n">
         <f aca="false">Model!AE184</f>
-        <v>61.3054809929673</v>
+        <v>61.4420444685691</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>